<commit_message>
Fixing Es translation in databooks
</commit_message>
<xml_diff>
--- a/inputs/es/LiST countries/AFG_databook.xlsx
+++ b/inputs/es/LiST countries/AFG_databook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tharindu.wickram\Desktop\Modeling\2025 studies\Nutrition\inputs\es\LiST countries\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4A6049B6-768A-4A4C-9400-A4F5BF34ABD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2FFDBDB-E1D6-4E8E-8CC6-49C3F762AE23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="20" windowWidth="19180" windowHeight="10180" tabRatio="961" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20" yWindow="20" windowWidth="19180" windowHeight="10180" tabRatio="961" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Entradas de población-año base" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="Distribución estado nutricional" sheetId="4" r:id="rId4"/>
     <sheet name="Distribución de lactancia" sheetId="5" r:id="rId5"/>
     <sheet name="Tendencias temporales" sheetId="6" r:id="rId6"/>
-    <sheet name="Variables económicas   " sheetId="7" r:id="rId7"/>
+    <sheet name="Variables económicas" sheetId="7" r:id="rId7"/>
     <sheet name="Paquetes de IYCF" sheetId="8" r:id="rId8"/>
     <sheet name="Tratamiento de la MAS" sheetId="9" r:id="rId9"/>
     <sheet name="Costo y cobertura del programa" sheetId="10" r:id="rId10"/>
@@ -20814,6 +20814,35 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="uneGi63yaLgZiuRTHC9TlVx0PCIeVisfQVWlzAxPigMQAfrva3e18eT+E+WPLYQgUyODrz7LSuBS71/swGbR0Q==" saltValue="8Cy9IsVLSynd8qdfIaw2lA==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <mergeCells count="45">
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="B36:B38"/>
+    <mergeCell ref="B92:B94"/>
+    <mergeCell ref="B114:B116"/>
+    <mergeCell ref="B45:B47"/>
+    <mergeCell ref="B22:B24"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="B78:B80"/>
+    <mergeCell ref="B108:B110"/>
+    <mergeCell ref="B55:B57"/>
+    <mergeCell ref="B84:B86"/>
+    <mergeCell ref="B89:B91"/>
+    <mergeCell ref="B154:B156"/>
+    <mergeCell ref="B64:B66"/>
+    <mergeCell ref="B95:B97"/>
+    <mergeCell ref="B25:B27"/>
+    <mergeCell ref="B125:B127"/>
+    <mergeCell ref="B131:B133"/>
+    <mergeCell ref="B31:B33"/>
+    <mergeCell ref="B75:B77"/>
+    <mergeCell ref="B81:B83"/>
+    <mergeCell ref="B72:B74"/>
+    <mergeCell ref="B134:B136"/>
+    <mergeCell ref="B151:B153"/>
+    <mergeCell ref="B148:B150"/>
+    <mergeCell ref="B137:B139"/>
+    <mergeCell ref="B128:B130"/>
+    <mergeCell ref="B142:B144"/>
     <mergeCell ref="B2:B4"/>
     <mergeCell ref="B117:B119"/>
     <mergeCell ref="B111:B113"/>
@@ -20830,35 +20859,6 @@
     <mergeCell ref="B98:B100"/>
     <mergeCell ref="B19:B21"/>
     <mergeCell ref="B28:B30"/>
-    <mergeCell ref="B154:B156"/>
-    <mergeCell ref="B64:B66"/>
-    <mergeCell ref="B95:B97"/>
-    <mergeCell ref="B25:B27"/>
-    <mergeCell ref="B125:B127"/>
-    <mergeCell ref="B131:B133"/>
-    <mergeCell ref="B31:B33"/>
-    <mergeCell ref="B75:B77"/>
-    <mergeCell ref="B81:B83"/>
-    <mergeCell ref="B72:B74"/>
-    <mergeCell ref="B134:B136"/>
-    <mergeCell ref="B151:B153"/>
-    <mergeCell ref="B148:B150"/>
-    <mergeCell ref="B137:B139"/>
-    <mergeCell ref="B128:B130"/>
-    <mergeCell ref="B142:B144"/>
-    <mergeCell ref="B5:B7"/>
-    <mergeCell ref="B36:B38"/>
-    <mergeCell ref="B92:B94"/>
-    <mergeCell ref="B114:B116"/>
-    <mergeCell ref="B45:B47"/>
-    <mergeCell ref="B22:B24"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="B78:B80"/>
-    <mergeCell ref="B108:B110"/>
-    <mergeCell ref="B55:B57"/>
-    <mergeCell ref="B84:B86"/>
-    <mergeCell ref="B89:B91"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -41619,16 +41619,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5de2aea6-bdc3-4e5f-b0ae-84d85b5764e4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100856A3DB4B0A5FF4A85E5854FA9B1BD84" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f77cb9dc30d15950233dec29875e7d3d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5de2aea6-bdc3-4e5f-b0ae-84d85b5764e4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c7972fb108f377c3e0c6a81e726e76be" ns2:_="">
     <xsd:import namespace="5de2aea6-bdc3-4e5f-b0ae-84d85b5764e4"/>
@@ -41812,6 +41802,16 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5de2aea6-bdc3-4e5f-b0ae-84d85b5764e4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -41822,16 +41822,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA1364B1-D0AC-4AFC-8837-019122E84913}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="5de2aea6-bdc3-4e5f-b0ae-84d85b5764e4"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{89AE9A51-FA73-431C-A4D5-36C1DFA1FEFD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -41849,6 +41839,16 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA1364B1-D0AC-4AFC-8837-019122E84913}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="5de2aea6-bdc3-4e5f-b0ae-84d85b5764e4"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BFA00B2B-FC7F-4ED6-BC3D-3DE83488E245}">
   <ds:schemaRefs>

</xml_diff>